<commit_message>
Atlas del Arboretum: fichas automaticas, catalogo, mapa, estadisticas, aves y datos
</commit_message>
<xml_diff>
--- a/data/Arboretum_Master.xlsx
+++ b/data/Arboretum_Master.xlsx
@@ -7469,7 +7469,7 @@
       </c>
       <c r="K32" s="5" t="inlineStr">
         <is>
-          <t>PechoAmarillo.JPG</t>
+          <t>Pechoamarillo.JPG</t>
         </is>
       </c>
       <c r="L32" s="8" t="n"/>
@@ -7881,7 +7881,7 @@
       </c>
       <c r="K42" s="5" t="inlineStr">
         <is>
-          <t>TyrannusSavana.jpg</t>
+          <t>Tyrannussavana.jpg</t>
         </is>
       </c>
       <c r="L42" s="8" t="n"/>
@@ -8041,7 +8041,7 @@
       </c>
       <c r="K46" s="5" t="inlineStr">
         <is>
-          <t>Tordorenegrido.JPG</t>
+          <t>TordoRenegrido.JPG</t>
         </is>
       </c>
       <c r="L46" s="8" t="n"/>

</xml_diff>